<commit_message>
Actualizar maestros de proveedores vía Telegram (0 nuevos, 1 corregidos)
Enviado por Telegram, aplicado sin revisión.
</commit_message>
<xml_diff>
--- a/proveedores.xlsx
+++ b/proveedores.xlsx
@@ -66338,10 +66338,10 @@
         </is>
       </c>
       <c r="B4990" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D4990" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4991">

</xml_diff>